<commit_message>
Ship platform OTP timed gates, guest/ops stack, and related production updates.
Adds Super Admin email/SMS OTP enable-disable windows, guest marketplace and privacy modules, admin/POS enhancements, and related API/SPA updates. CD workflow YAMLs deferred pending workflow-scope token.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/qa/export/excel/CREDENTIALS_LOG.xlsx
+++ b/docs/qa/export/excel/CREDENTIALS_LOG.xlsx
@@ -125,10 +125,10 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Waiter URL</t>
-  </si>
-  <si>
-    <t>https://waiter.cullinos.com</t>
+    <t>Waiter app</t>
+  </si>
+  <si>
+    <t>Cullinos Waiter Android</t>
   </si>
   <si>
     <t>Optional Cashier</t>

</xml_diff>